<commit_message>
Enrich with LunarCrush-verified follower counts (YouTube + X)
- Connected LunarCrush MCP; pulled live verified follower counts for ~35 creators
  across YouTube and X (tagged '(LunarCrush 2026-07-19)' in followers field)
- Recomputed tiers/pricing/scores from real numbers; corrected estimates
  (Bouchonnoir 2,850; Aiden Gambles 5,930; PokiChloe 136k; Watchfinder 1.17M;
  Nico Leonard 2.06M; Lady Luck HQ 1.2M; Vegas Matt 1.61M; etc.)
- README documents coverage: YouTube/X verified; Instagram returns empty (still
  estimate/paste); Kick/Twitch not covered (YT number is a floor for stream-first
  gamblers). Fixed a substring false-positive (Andrew Morgan vs Watchfinder)
- Regenerated xlsx + pdf

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Uk2hYJEbFcdAHcmepwjE9x
</commit_message>
<xml_diff>
--- a/research/GemBreak_Influencer_Lists.xlsx
+++ b/research/GemBreak_Influencer_Lists.xlsx
@@ -881,12 +881,12 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>OneEyedGregg</t>
+          <t>Fruity Slots (Josh/Jamie/Scottie)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>case-opening/mystery-box</t>
+          <t>gambling-casino</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -901,47 +901,47 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Kick ~14.9k (snippet)</t>
+          <t>78,700 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="G4" s="4" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>Kick https://kick.com/oneeyedgregg ; YouTube https://www.youtube.com/@Oneeyedgregg ; Twitch https://www.twitch.tv/oneeyedgregg ; X https://x.com/oneeyedgregg</t>
+          <t>YouTube @FruitySlots</t>
         </is>
       </c>
       <c r="I4" s="4" t="inlineStr">
         <is>
-          <t>none (oeg.gg hub)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J4" s="4" t="inlineStr">
         <is>
-          <t>4.3</t>
+          <t>4.4</t>
         </is>
       </c>
       <c r="K4" s="4" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="M4" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="N4" s="5" t="inlineStr">
         <is>
-          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O4" s="4" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>lacedupny (Laced Up Worldwide)</t>
+          <t>Rydurz</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -983,22 +983,22 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>~20k IG ESTIMATE (pikdo mirror 2026-07-18)</t>
+          <t>12,801 X (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>Kick</t>
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr">
         <is>
-          <t>Instagram https://www.instagram.com/lacedupny/</t>
+          <t>Kick https://kick.com/rydurz ; X https://x.com/rydurz</t>
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr">
         <is>
-          <t>retail store (multi-location)</t>
+          <t>none (coderydurz.com hub)</t>
         </is>
       </c>
       <c r="J5" s="6" t="inlineStr">
@@ -1045,7 +1045,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Rydurz</t>
+          <t>OneEyedGregg</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
@@ -1065,7 +1065,7 @@
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>Kick ~24.2k (Sept-2025 snippet)</t>
+          <t>Kick ~14.9k (snippet)</t>
         </is>
       </c>
       <c r="G6" s="4" t="inlineStr">
@@ -1075,12 +1075,12 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>Kick https://kick.com/rydurz ; X https://x.com/rydurz</t>
+          <t>Kick https://kick.com/oneeyedgregg ; YouTube https://www.youtube.com/@Oneeyedgregg ; Twitch https://www.twitch.tv/oneeyedgregg ; X https://x.com/oneeyedgregg</t>
         </is>
       </c>
       <c r="I6" s="4" t="inlineStr">
         <is>
-          <t>none (coderydurz.com hub)</t>
+          <t>none (oeg.gg hub)</t>
         </is>
       </c>
       <c r="J6" s="4" t="inlineStr">
@@ -1127,7 +1127,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Jules (Julsy)</t>
+          <t>lacedupny (Laced Up Worldwide)</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -1147,22 +1147,22 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>~20k IG ESTIMATE (pikdo mirror 2026-07-18)</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
-          <t>YouTube https://www.youtube.com/channel/UCrUFQtoCMdDZ06whZQodFuA ; X https://x.com/JulsyCS ; Kick https://kick.com/JULSY</t>
+          <t>Instagram https://www.instagram.com/lacedupny/</t>
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>retail store (multi-location)</t>
         </is>
       </c>
       <c r="J7" s="6" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>RobZn</t>
+          <t>Jules (Julsy)</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
@@ -1234,12 +1234,12 @@
       </c>
       <c r="G8" s="4" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Kick https://kick.com/robznnncs</t>
+          <t>YouTube https://www.youtube.com/channel/UCrUFQtoCMdDZ06whZQodFuA ; X https://x.com/JulsyCS ; Kick https://kick.com/JULSY</t>
         </is>
       </c>
       <c r="I8" s="4" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>@the_happy_budget</t>
+          <t>RobZn</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1316,12 +1316,12 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Kick</t>
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@the_happy_budget</t>
+          <t>Kick https://kick.com/robznnncs</t>
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>@winonakicks</t>
+          <t>@the_happy_budget</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="H10" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@winonakicks</t>
+          <t>https://www.tiktok.com/@the_happy_budget</t>
         </is>
       </c>
       <c r="I10" s="4" t="inlineStr">
@@ -1455,17 +1455,17 @@
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Maria Ho</t>
+          <t>@winonakicks</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>gambling-casino</t>
+          <t>case-opening/mystery-box</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -1475,22 +1475,22 @@
       </c>
       <c r="F11" s="6" t="inlineStr">
         <is>
-          <t>mid-macro ESTIMATE</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G11" s="6" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
-          <t>IG https://instagram.com/maria_ho</t>
+          <t>https://www.tiktok.com/@winonakicks</t>
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>https://www.mariaho.com</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J11" s="6" t="inlineStr">
@@ -1500,32 +1500,32 @@
       </c>
       <c r="K11" s="6" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="M11" s="6" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N11" s="7" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; reachable via site/store</t>
+          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O11" s="6" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="P11" s="6" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
     </row>
@@ -1537,7 +1537,7 @@
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Jonathan Little</t>
+          <t>Maria Ho</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
@@ -1557,7 +1557,7 @@
       </c>
       <c r="F12" s="4" t="inlineStr">
         <is>
-          <t>mid ESTIMATE</t>
+          <t>mid-macro ESTIMATE</t>
         </is>
       </c>
       <c r="G12" s="4" t="inlineStr">
@@ -1567,12 +1567,12 @@
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>IG https://instagram.com/jonathanlittlepoker ; site pokercoaching.com</t>
+          <t>IG https://instagram.com/maria_ho</t>
         </is>
       </c>
       <c r="I12" s="4" t="inlineStr">
         <is>
-          <t>https://pokercoaching.com</t>
+          <t>https://www.mariaho.com</t>
         </is>
       </c>
       <c r="J12" s="4" t="inlineStr">
@@ -1619,17 +1619,17 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>mysterypacks.de</t>
+          <t>Jonathan Little</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>case-opening/mystery-box</t>
+          <t>gambling-casino</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>micro</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -1639,22 +1639,22 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>52.1k TikTok (2026-07-18)</t>
+          <t>mid ESTIMATE</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@mysterypacks.de</t>
+          <t>IG https://instagram.com/jonathanlittlepoker ; site pokercoaching.com</t>
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>https://pokercoaching.com</t>
         </is>
       </c>
       <c r="J13" s="6" t="inlineStr">
@@ -1664,32 +1664,32 @@
       </c>
       <c r="K13" s="6" t="inlineStr">
         <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="M13" s="6" t="inlineStr">
+        <is>
           <t>4.0</t>
         </is>
       </c>
-      <c r="L13" s="6" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
-      <c r="M13" s="6" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="N13" s="7" t="inlineStr">
         <is>
-          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; reachable via site/store</t>
         </is>
       </c>
       <c r="O13" s="6" t="inlineStr">
         <is>
-          <t>$175-1,500</t>
+          <t>$1,500-6,000</t>
         </is>
       </c>
       <c r="P13" s="6" t="inlineStr">
         <is>
-          <t>$4,400-27,000</t>
+          <t>$27,000-90,000</t>
         </is>
       </c>
     </row>
@@ -1701,7 +1701,7 @@
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>Svensk Drama</t>
+          <t>mysterypacks.de</t>
         </is>
       </c>
       <c r="C14" s="4" t="inlineStr">
@@ -1721,17 +1721,17 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>~67.8k SUBS (2026-06-24, single-source)</t>
+          <t>52.1k TikTok (2026-07-18)</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>YouTube https://www.youtube.com/@SvenskDrama</t>
+          <t>TikTok https://www.tiktok.com/@mysterypacks.de</t>
         </is>
       </c>
       <c r="I14" s="4" t="inlineStr">
@@ -1783,7 +1783,7 @@
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>unboxdisneypinco</t>
+          <t>Svensk Drama</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -1793,7 +1793,7 @@
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>nano</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
@@ -1803,17 +1803,17 @@
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>2,751 IG (2026-07-18)</t>
+          <t>~67.8k SUBS (2026-06-24, single-source)</t>
         </is>
       </c>
       <c r="G15" s="6" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr">
         <is>
-          <t>Instagram https://www.instagram.com/unboxdisneypinco/</t>
+          <t>YouTube https://www.youtube.com/@SvenskDrama</t>
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="J15" s="6" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>4.3</t>
         </is>
       </c>
       <c r="K15" s="6" t="inlineStr">
@@ -1848,12 +1848,12 @@
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>$50-300</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="P15" s="6" t="inlineStr">
         <is>
-          <t>$450-4,400</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
     </row>
@@ -1865,7 +1865,7 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>CrimsonYT</t>
+          <t>GW1917</t>
         </is>
       </c>
       <c r="C16" s="4" t="inlineStr">
@@ -1875,7 +1875,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>nano-micro</t>
+          <t>nano</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>~5k YT SUBS (SERP)</t>
+          <t>453 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1895,12 +1895,12 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>YouTube https://www.youtube.com/channel/UCI2grI-9aZh9kyuPxWAFvxg ; X https://x.com/CrimsonYT101</t>
+          <t>YouTube https://www.youtube.com/@GW1917gaming</t>
         </is>
       </c>
       <c r="I16" s="4" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>none (gw1917gaming.com)</t>
         </is>
       </c>
       <c r="J16" s="4" t="inlineStr">
@@ -1930,12 +1930,12 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>$175-1,500</t>
+          <t>$50-300</t>
         </is>
       </c>
       <c r="P16" s="4" t="inlineStr">
         <is>
-          <t>$4,400-27,000</t>
+          <t>$450-4,400</t>
         </is>
       </c>
     </row>
@@ -1947,17 +1947,17 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Slot Squad</t>
+          <t>unboxdisneypinco</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>gambling-casino</t>
+          <t>case-opening/mystery-box</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>micro</t>
+          <t>nano</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
@@ -1967,7 +1967,7 @@
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>~16k IG</t>
+          <t>2,751 IG (2026-07-18)</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -1977,7 +1977,7 @@
       </c>
       <c r="H17" s="7" t="inlineStr">
         <is>
-          <t>IG https://instagram.com/theslotsquad (16k)</t>
+          <t>Instagram https://www.instagram.com/unboxdisneypinco/</t>
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr">
@@ -1992,32 +1992,32 @@
       </c>
       <c r="K17" s="6" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="M17" s="6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O17" s="6" t="inlineStr">
         <is>
-          <t>$175-1,500</t>
+          <t>$50-300</t>
         </is>
       </c>
       <c r="P17" s="6" t="inlineStr">
         <is>
-          <t>$4,400-27,000</t>
+          <t>$450-4,400</t>
         </is>
       </c>
     </row>
@@ -2029,17 +2029,17 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>clvkingbets</t>
+          <t>Bouchonnoir</t>
         </is>
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>sports-betting</t>
+          <t>case-opening/mystery-box</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>micro</t>
+          <t>nano</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
@@ -2049,22 +2049,22 @@
       </c>
       <c r="F18" s="4" t="inlineStr">
         <is>
-          <t>~18.8k</t>
+          <t>2,850 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>TikTok @clvkingbets (18.8k)</t>
+          <t>YouTube https://www.youtube.com/@Bouchonnoir</t>
         </is>
       </c>
       <c r="I18" s="4" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>none (bouchonnoir.gg hub)</t>
         </is>
       </c>
       <c r="J18" s="4" t="inlineStr">
@@ -2074,32 +2074,32 @@
       </c>
       <c r="K18" s="4" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="M18" s="4" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N18" s="5" t="inlineStr">
         <is>
-          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>$175-1,500</t>
+          <t>$50-300</t>
         </is>
       </c>
       <c r="P18" s="4" t="inlineStr">
         <is>
-          <t>$4,400-27,000</t>
+          <t>$450-4,400</t>
         </is>
       </c>
     </row>
@@ -2111,17 +2111,17 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>gurusportsbetting</t>
+          <t>CrimsonYT</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>sports-betting</t>
+          <t>case-opening/mystery-box</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>micro</t>
+          <t>nano-micro</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -2131,17 +2131,17 @@
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>~19.3k</t>
+          <t>~5k YT SUBS (SERP)</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H19" s="7" t="inlineStr">
         <is>
-          <t>TikTok @gurusportsbetting (19.3k)</t>
+          <t>YouTube https://www.youtube.com/channel/UCI2grI-9aZh9kyuPxWAFvxg ; X https://x.com/CrimsonYT101</t>
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr">
@@ -2156,22 +2156,22 @@
       </c>
       <c r="K19" s="6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="M19" s="6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N19" s="7" t="inlineStr">
         <is>
-          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O19" s="6" t="inlineStr">
@@ -2193,17 +2193,17 @@
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>lucyburdge1</t>
+          <t>Sloth (SlothCSGO)</t>
         </is>
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>sports-betting</t>
+          <t>case-opening/mystery-box</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>micro</t>
+          <t>nano</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -2213,22 +2213,22 @@
       </c>
       <c r="F20" s="4" t="inlineStr">
         <is>
-          <t>~19.5k</t>
+          <t>5,880 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="G20" s="4" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>TikTok @lucyburdge1 (19.5k)</t>
+          <t>YouTube https://www.youtube.com/@SlothCSGO ; X https://x.com/slothhcsgo</t>
         </is>
       </c>
       <c r="I20" s="4" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>none (slothrewards.com hub)</t>
         </is>
       </c>
       <c r="J20" s="4" t="inlineStr">
@@ -2238,32 +2238,32 @@
       </c>
       <c r="K20" s="4" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="M20" s="4" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N20" s="5" t="inlineStr">
         <is>
-          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>$175-1,500</t>
+          <t>$50-300</t>
         </is>
       </c>
       <c r="P20" s="4" t="inlineStr">
         <is>
-          <t>$4,400-27,000</t>
+          <t>$450-4,400</t>
         </is>
       </c>
     </row>
@@ -2275,17 +2275,17 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t>brucie.sports</t>
+          <t>Aiden Gambles</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>sports-betting</t>
+          <t>case-opening/mystery-box</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>micro</t>
+          <t>nano</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
@@ -2295,22 +2295,22 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>~23.9k</t>
+          <t>5,930 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H21" s="7" t="inlineStr">
         <is>
-          <t>TikTok @brucie.sports (23.9k)</t>
+          <t>YouTube https://www.youtube.com/@AidenGambles ; X https://x.com/aiden_gambles</t>
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>none (Discord community)</t>
         </is>
       </c>
       <c r="J21" s="6" t="inlineStr">
@@ -2320,32 +2320,32 @@
       </c>
       <c r="K21" s="6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="L21" s="6" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="M21" s="6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O21" s="6" t="inlineStr">
         <is>
-          <t>$175-1,500</t>
+          <t>$50-300</t>
         </is>
       </c>
       <c r="P21" s="6" t="inlineStr">
         <is>
-          <t>$4,400-27,000</t>
+          <t>$450-4,400</t>
         </is>
       </c>
     </row>
@@ -2357,12 +2357,12 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>codycoverspreads</t>
+          <t>Slot Squad</t>
         </is>
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>sports-betting</t>
+          <t>gambling-casino</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -2377,17 +2377,17 @@
       </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
-          <t>~27.2k</t>
+          <t>~16k IG</t>
         </is>
       </c>
       <c r="G22" s="4" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="H22" s="5" t="inlineStr">
         <is>
-          <t>TikTok @codycoverspreads (27.2k)</t>
+          <t>IG https://instagram.com/theslotsquad (16k)</t>
         </is>
       </c>
       <c r="I22" s="4" t="inlineStr">
@@ -2402,22 +2402,22 @@
       </c>
       <c r="K22" s="4" t="inlineStr">
         <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
           <t>2.0</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="M22" s="4" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
       <c r="N22" s="5" t="inlineStr">
         <is>
-          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O22" s="4" t="inlineStr">
@@ -2439,12 +2439,12 @@
       </c>
       <c r="B23" s="6" t="inlineStr">
         <is>
-          <t>SweetFlips (group)</t>
+          <t>clvkingbets</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>gambling-casino</t>
+          <t>sports-betting</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
@@ -2459,17 +2459,17 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>~32k Kick</t>
+          <t>~18.8k</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H23" s="7" t="inlineStr">
         <is>
-          <t>Kick @SweetFlips (Dennylo, Damil, Jacko, Pingue, Baka, Motion, Blendz)</t>
+          <t>TikTok @clvkingbets (18.8k)</t>
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr">
@@ -2484,14 +2484,14 @@
       </c>
       <c r="K23" s="6" t="inlineStr">
         <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
           <t>3.0</t>
         </is>
       </c>
-      <c r="L23" s="6" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
       <c r="M23" s="6" t="inlineStr">
         <is>
           <t>2.0</t>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O23" s="6" t="inlineStr">
@@ -2521,17 +2521,17 @@
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Aiden Gambles</t>
+          <t>gurusportsbetting</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>case-opening/mystery-box</t>
+          <t>sports-betting</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>micro-mid</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -2541,22 +2541,22 @@
       </c>
       <c r="F24" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>~19.3k</t>
         </is>
       </c>
       <c r="G24" s="4" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H24" s="5" t="inlineStr">
         <is>
-          <t>YouTube https://www.youtube.com/@AidenGambles ; X https://x.com/aiden_gambles</t>
+          <t>TikTok @gurusportsbetting (19.3k)</t>
         </is>
       </c>
       <c r="I24" s="4" t="inlineStr">
         <is>
-          <t>none (Discord community)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J24" s="4" t="inlineStr">
@@ -2566,32 +2566,32 @@
       </c>
       <c r="K24" s="4" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="M24" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="N24" s="5" t="inlineStr">
         <is>
-          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O24" s="4" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="P24" s="4" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
     </row>
@@ -2603,17 +2603,17 @@
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>Bouchonnoir</t>
+          <t>lucyburdge1</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>case-opening/mystery-box</t>
+          <t>sports-betting</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>micro-mid</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -2623,22 +2623,22 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>~19.5k</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr">
         <is>
-          <t>YouTube https://www.youtube.com/@Bouchonnoir</t>
+          <t>TikTok @lucyburdge1 (19.5k)</t>
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr">
         <is>
-          <t>none (bouchonnoir.gg hub)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J25" s="6" t="inlineStr">
@@ -2648,32 +2648,32 @@
       </c>
       <c r="K25" s="6" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L25" s="6" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="M25" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O25" s="6" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="P25" s="6" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
     </row>
@@ -2685,17 +2685,17 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>GW1917</t>
+          <t>brucie.sports</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>case-opening/mystery-box</t>
+          <t>sports-betting</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>micro-mid</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -2705,22 +2705,22 @@
       </c>
       <c r="F26" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>~23.9k</t>
         </is>
       </c>
       <c r="G26" s="4" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr">
         <is>
-          <t>YouTube https://www.youtube.com/@GW1917gaming</t>
+          <t>TikTok @brucie.sports (23.9k)</t>
         </is>
       </c>
       <c r="I26" s="4" t="inlineStr">
         <is>
-          <t>none (gw1917gaming.com)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J26" s="4" t="inlineStr">
@@ -2730,32 +2730,32 @@
       </c>
       <c r="K26" s="4" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="M26" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="N26" s="5" t="inlineStr">
         <is>
-          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O26" s="4" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="P26" s="4" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
     </row>
@@ -2767,17 +2767,17 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Sloth (SlothCSGO)</t>
+          <t>codycoverspreads</t>
         </is>
       </c>
       <c r="C27" s="6" t="inlineStr">
         <is>
-          <t>case-opening/mystery-box</t>
+          <t>sports-betting</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>micro-mid</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
@@ -2787,22 +2787,22 @@
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>~27.2k</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr">
         <is>
-          <t>YouTube https://www.youtube.com/@SlothCSGO ; X https://x.com/slothhcsgo</t>
+          <t>TikTok @codycoverspreads (27.2k)</t>
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr">
         <is>
-          <t>none (slothrewards.com hub)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J27" s="6" t="inlineStr">
@@ -2812,32 +2812,32 @@
       </c>
       <c r="K27" s="6" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="L27" s="6" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="M27" s="6" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O27" s="6" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="P27" s="6" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
     </row>
@@ -2849,17 +2849,17 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>TylerPlaysLive</t>
+          <t>SweetFlips (group)</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>case-opening/mystery-box</t>
+          <t>gambling-casino</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>micro-mid</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -2869,22 +2869,22 @@
       </c>
       <c r="F28" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>~32k Kick</t>
         </is>
       </c>
       <c r="G28" s="4" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Kick</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>YouTube https://www.youtube.com/@tylerplayslive26 ; TikTok https://www.tiktok.com/@tylerplaylive ; X https://x.com/tylerplayslive ; Kick https://kick.com/tylerplayslive</t>
+          <t>Kick @SweetFlips (Dennylo, Damil, Jacko, Pingue, Baka, Motion, Blendz)</t>
         </is>
       </c>
       <c r="I28" s="4" t="inlineStr">
         <is>
-          <t>none (BlissBox LLC FB page)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J28" s="4" t="inlineStr">
@@ -2894,32 +2894,32 @@
       </c>
       <c r="K28" s="4" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="M28" s="4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="N28" s="5" t="inlineStr">
         <is>
-          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="P28" s="4" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
     </row>
@@ -2931,7 +2931,7 @@
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t>emilyyyrosess</t>
+          <t>TylerPlaysLive</t>
         </is>
       </c>
       <c r="C29" s="6" t="inlineStr">
@@ -2941,7 +2941,7 @@
       </c>
       <c r="D29" s="6" t="inlineStr">
         <is>
-          <t>nano-micro</t>
+          <t>micro-mid</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
@@ -2956,17 +2956,17 @@
       </c>
       <c r="G29" s="6" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H29" s="7" t="inlineStr">
         <is>
-          <t>Instagram https://www.instagram.com/emilyyyrosess/</t>
+          <t>YouTube https://www.youtube.com/@tylerplayslive26 ; TikTok https://www.tiktok.com/@tylerplaylive ; X https://x.com/tylerplayslive ; Kick https://kick.com/tylerplayslive</t>
         </is>
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>none (BlissBox LLC FB page)</t>
         </is>
       </c>
       <c r="J29" s="6" t="inlineStr">
@@ -2996,12 +2996,12 @@
       </c>
       <c r="O29" s="6" t="inlineStr">
         <is>
-          <t>$175-1,500</t>
+          <t>$1,500-6,000</t>
         </is>
       </c>
       <c r="P29" s="6" t="inlineStr">
         <is>
-          <t>$4,400-27,000</t>
+          <t>$27,000-90,000</t>
         </is>
       </c>
     </row>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>golddigger_5</t>
+          <t>emilyyyrosess</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -3038,12 +3038,12 @@
       </c>
       <c r="G30" s="4" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@golddigger_5</t>
+          <t>Instagram https://www.instagram.com/emilyyyrosess/</t>
         </is>
       </c>
       <c r="I30" s="4" t="inlineStr">
@@ -3095,7 +3095,7 @@
       </c>
       <c r="B31" s="6" t="inlineStr">
         <is>
-          <t>hypedropcrazybattles</t>
+          <t>golddigger_5</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -3125,7 +3125,7 @@
       </c>
       <c r="H31" s="7" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@hypedropcrazybattles</t>
+          <t>TikTok https://www.tiktok.com/@golddigger_5</t>
         </is>
       </c>
       <c r="I31" s="6" t="inlineStr">
@@ -3177,7 +3177,7 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>Sebknowsbest</t>
+          <t>hypedropcrazybattles</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -3207,7 +3207,7 @@
       </c>
       <c r="H32" s="5" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@sebknowsbest</t>
+          <t>TikTok https://www.tiktok.com/@hypedropcrazybattles</t>
         </is>
       </c>
       <c r="I32" s="4" t="inlineStr">
@@ -3259,7 +3259,7 @@
       </c>
       <c r="B33" s="6" t="inlineStr">
         <is>
-          <t>tshockz22</t>
+          <t>Sebknowsbest</t>
         </is>
       </c>
       <c r="C33" s="6" t="inlineStr">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="H33" s="7" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@tshockz22</t>
+          <t>TikTok https://www.tiktok.com/@sebknowsbest</t>
         </is>
       </c>
       <c r="I33" s="6" t="inlineStr">
@@ -3341,17 +3341,17 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>Brian Christopher (BCSlots)</t>
+          <t>tshockz22</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>gambling-casino</t>
+          <t>case-opening/mystery-box</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>nano-micro</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -3361,17 +3361,17 @@
       </c>
       <c r="F34" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G34" s="4" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr">
         <is>
-          <t>YouTube @BrianChristopherSlots ; site bcslots.com</t>
+          <t>TikTok https://www.tiktok.com/@tshockz22</t>
         </is>
       </c>
       <c r="I34" s="4" t="inlineStr">
@@ -3386,32 +3386,32 @@
       </c>
       <c r="K34" s="4" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="M34" s="4" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N34" s="5" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; macro reach (higher cost); reachable via site/store</t>
+          <t>real-money case/box gambling - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O34" s="4" t="inlineStr">
         <is>
-          <t>$6,000-30,000</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="P34" s="4" t="inlineStr">
         <is>
-          <t>$90,000-700,000+</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
     </row>
@@ -3423,7 +3423,7 @@
       </c>
       <c r="B35" s="6" t="inlineStr">
         <is>
-          <t>LetsGiveItASpin (Kim Hultman)</t>
+          <t>Brian Christopher (BCSlots)</t>
         </is>
       </c>
       <c r="C35" s="6" t="inlineStr">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="D35" s="6" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>macro</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
@@ -3443,7 +3443,7 @@
       </c>
       <c r="F35" s="6" t="inlineStr">
         <is>
-          <t>mid-macro</t>
+          <t>macro</t>
         </is>
       </c>
       <c r="G35" s="6" t="inlineStr">
@@ -3453,7 +3453,7 @@
       </c>
       <c r="H35" s="7" t="inlineStr">
         <is>
-          <t>YouTube @LetsGiveItASpin</t>
+          <t>YouTube @BrianChristopherSlots ; site bcslots.com</t>
         </is>
       </c>
       <c r="I35" s="6" t="inlineStr">
@@ -3478,22 +3478,22 @@
       </c>
       <c r="M35" s="6" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; macro reach (higher cost); reachable via site/store</t>
         </is>
       </c>
       <c r="O35" s="6" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$6,000-30,000</t>
         </is>
       </c>
       <c r="P35" s="6" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$90,000-700,000+</t>
         </is>
       </c>
     </row>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>CasinoGrounds</t>
+          <t>LetsGiveItASpin (Kim Hultman)</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -3525,7 +3525,7 @@
       </c>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>mid-macro</t>
         </is>
       </c>
       <c r="G36" s="4" t="inlineStr">
@@ -3535,7 +3535,7 @@
       </c>
       <c r="H36" s="5" t="inlineStr">
         <is>
-          <t>YouTube (CasinoGrounds)</t>
+          <t>YouTube @LetsGiveItASpin</t>
         </is>
       </c>
       <c r="I36" s="4" t="inlineStr">
@@ -3669,17 +3669,17 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>Fruity Slots (Josh/Jamie/Scottie)</t>
+          <t>BenderWins Sports Betting</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>gambling-casino</t>
+          <t>sports-betting</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
@@ -3689,17 +3689,17 @@
       </c>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>micro ESTIMATE</t>
         </is>
       </c>
       <c r="G38" s="4" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>YouTube @FruitySlots</t>
+          <t>TikTok @BenderWinsSportsBetting</t>
         </is>
       </c>
       <c r="I38" s="4" t="inlineStr">
@@ -3714,32 +3714,32 @@
       </c>
       <c r="K38" s="4" t="inlineStr">
         <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
           <t>3.0</t>
         </is>
       </c>
-      <c r="L38" s="4" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
       <c r="M38" s="4" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="N38" s="5" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; contact needs enrichment</t>
+          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O38" s="4" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="P38" s="4" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
     </row>
@@ -3751,12 +3751,12 @@
       </c>
       <c r="B39" s="6" t="inlineStr">
         <is>
-          <t>BenderWins Sports Betting</t>
+          <t>Brett Stern</t>
         </is>
       </c>
       <c r="C39" s="6" t="inlineStr">
         <is>
-          <t>sports-betting</t>
+          <t>gambling-casino</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
@@ -3776,12 +3776,12 @@
       </c>
       <c r="G39" s="6" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="H39" s="7" t="inlineStr">
         <is>
-          <t>TikTok @BenderWinsSportsBetting</t>
+          <t>IG (gambling)</t>
         </is>
       </c>
       <c r="I39" s="6" t="inlineStr">
@@ -3796,22 +3796,22 @@
       </c>
       <c r="K39" s="6" t="inlineStr">
         <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M39" s="6" t="inlineStr">
+        <is>
           <t>2.0</t>
         </is>
       </c>
-      <c r="L39" s="6" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="M39" s="6" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
       <c r="N39" s="7" t="inlineStr">
         <is>
-          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O39" s="6" t="inlineStr">
@@ -3833,12 +3833,12 @@
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>Brett Stern</t>
+          <t>weberbets</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>gambling-casino</t>
+          <t>sports-betting</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -3853,17 +3853,17 @@
       </c>
       <c r="F40" s="4" t="inlineStr">
         <is>
-          <t>micro ESTIMATE</t>
+          <t>~40.4k</t>
         </is>
       </c>
       <c r="G40" s="4" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr">
         <is>
-          <t>IG (gambling)</t>
+          <t>TikTok @weberbets (40.4k)</t>
         </is>
       </c>
       <c r="I40" s="4" t="inlineStr">
@@ -3878,14 +3878,14 @@
       </c>
       <c r="K40" s="4" t="inlineStr">
         <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
           <t>3.0</t>
         </is>
       </c>
-      <c r="L40" s="4" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
       <c r="M40" s="4" t="inlineStr">
         <is>
           <t>2.0</t>
@@ -3893,7 +3893,7 @@
       </c>
       <c r="N40" s="5" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O40" s="4" t="inlineStr">
@@ -3915,12 +3915,12 @@
       </c>
       <c r="B41" s="6" t="inlineStr">
         <is>
-          <t>weberbets</t>
+          <t>Heart of Vegas Slots</t>
         </is>
       </c>
       <c r="C41" s="6" t="inlineStr">
         <is>
-          <t>sports-betting</t>
+          <t>gambling-casino</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
@@ -3935,17 +3935,17 @@
       </c>
       <c r="F41" s="6" t="inlineStr">
         <is>
-          <t>~40.4k</t>
+          <t>~47k IG</t>
         </is>
       </c>
       <c r="G41" s="6" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr">
         <is>
-          <t>TikTok @weberbets (40.4k)</t>
+          <t>IG https://instagram.com/heartofvegasslots (47k)</t>
         </is>
       </c>
       <c r="I41" s="6" t="inlineStr">
@@ -3975,7 +3975,7 @@
       </c>
       <c r="N41" s="7" t="inlineStr">
         <is>
-          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O41" s="6" t="inlineStr">
@@ -3997,12 +3997,12 @@
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>Heart of Vegas Slots</t>
+          <t>takingthepoints</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>gambling-casino</t>
+          <t>sports-betting</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -4017,17 +4017,17 @@
       </c>
       <c r="F42" s="4" t="inlineStr">
         <is>
-          <t>~47k IG</t>
+          <t>~60.4k</t>
         </is>
       </c>
       <c r="G42" s="4" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>IG https://instagram.com/heartofvegasslots (47k)</t>
+          <t>TikTok @takingthepoints (60.4k)</t>
         </is>
       </c>
       <c r="I42" s="4" t="inlineStr">
@@ -4057,7 +4057,7 @@
       </c>
       <c r="N42" s="5" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O42" s="4" t="inlineStr">
@@ -4079,12 +4079,12 @@
       </c>
       <c r="B43" s="6" t="inlineStr">
         <is>
-          <t>takingthepoints</t>
+          <t>jommypogs</t>
         </is>
       </c>
       <c r="C43" s="6" t="inlineStr">
         <is>
-          <t>sports-betting</t>
+          <t>gambling-casino</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
@@ -4099,7 +4099,7 @@
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>~60.4k</t>
+          <t>~61.4k TT</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -4109,7 +4109,7 @@
       </c>
       <c r="H43" s="7" t="inlineStr">
         <is>
-          <t>TikTok @takingthepoints (60.4k)</t>
+          <t>TikTok @jommypogs</t>
         </is>
       </c>
       <c r="I43" s="6" t="inlineStr">
@@ -4124,22 +4124,22 @@
       </c>
       <c r="K43" s="6" t="inlineStr">
         <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M43" s="6" t="inlineStr">
+        <is>
           <t>2.0</t>
         </is>
       </c>
-      <c r="L43" s="6" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="M43" s="6" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
       <c r="N43" s="7" t="inlineStr">
         <is>
-          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O43" s="6" t="inlineStr">
@@ -4161,7 +4161,7 @@
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>jommypogs</t>
+          <t>jstros_</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -4181,7 +4181,7 @@
       </c>
       <c r="F44" s="4" t="inlineStr">
         <is>
-          <t>~61.4k TT</t>
+          <t>~62.1k TT</t>
         </is>
       </c>
       <c r="G44" s="4" t="inlineStr">
@@ -4191,7 +4191,7 @@
       </c>
       <c r="H44" s="5" t="inlineStr">
         <is>
-          <t>TikTok @jommypogs</t>
+          <t>TikTok @jstros_</t>
         </is>
       </c>
       <c r="I44" s="4" t="inlineStr">
@@ -4243,7 +4243,7 @@
       </c>
       <c r="B45" s="6" t="inlineStr">
         <is>
-          <t>jstros_</t>
+          <t>binkyloveslots</t>
         </is>
       </c>
       <c r="C45" s="6" t="inlineStr">
@@ -4273,7 +4273,7 @@
       </c>
       <c r="H45" s="7" t="inlineStr">
         <is>
-          <t>TikTok @jstros_</t>
+          <t>TikTok @binkyloveslots</t>
         </is>
       </c>
       <c r="I45" s="6" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>binkyloveslots</t>
+          <t>ahmed_elpoker</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -4345,7 +4345,7 @@
       </c>
       <c r="F46" s="4" t="inlineStr">
         <is>
-          <t>~62.1k TT</t>
+          <t>~62.3k TT</t>
         </is>
       </c>
       <c r="G46" s="4" t="inlineStr">
@@ -4355,7 +4355,7 @@
       </c>
       <c r="H46" s="5" t="inlineStr">
         <is>
-          <t>TikTok @binkyloveslots</t>
+          <t>TikTok @ahmed_elpoker</t>
         </is>
       </c>
       <c r="I46" s="4" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="B47" s="6" t="inlineStr">
         <is>
-          <t>ahmed_elpoker</t>
+          <t>thadrunkgambler</t>
         </is>
       </c>
       <c r="C47" s="6" t="inlineStr">
@@ -4427,7 +4427,7 @@
       </c>
       <c r="F47" s="6" t="inlineStr">
         <is>
-          <t>~62.3k TT</t>
+          <t>~64k TT</t>
         </is>
       </c>
       <c r="G47" s="6" t="inlineStr">
@@ -4437,7 +4437,7 @@
       </c>
       <c r="H47" s="7" t="inlineStr">
         <is>
-          <t>TikTok @ahmed_elpoker</t>
+          <t>TikTok @thadrunkgambler</t>
         </is>
       </c>
       <c r="I47" s="6" t="inlineStr">
@@ -4489,7 +4489,7 @@
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>thadrunkgambler</t>
+          <t>thequeenofmedia</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -4509,7 +4509,7 @@
       </c>
       <c r="F48" s="4" t="inlineStr">
         <is>
-          <t>~64k TT</t>
+          <t>~79.8k TT</t>
         </is>
       </c>
       <c r="G48" s="4" t="inlineStr">
@@ -4519,7 +4519,7 @@
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>TikTok @thadrunkgambler</t>
+          <t>TikTok @thequeenofmedia</t>
         </is>
       </c>
       <c r="I48" s="4" t="inlineStr">
@@ -4571,12 +4571,12 @@
       </c>
       <c r="B49" s="6" t="inlineStr">
         <is>
-          <t>thequeenofmedia</t>
+          <t>erinkatedolan</t>
         </is>
       </c>
       <c r="C49" s="6" t="inlineStr">
         <is>
-          <t>gambling-casino</t>
+          <t>sports-betting</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
@@ -4591,7 +4591,7 @@
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>~79.8k TT</t>
+          <t>~81.3k</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
@@ -4601,7 +4601,7 @@
       </c>
       <c r="H49" s="7" t="inlineStr">
         <is>
-          <t>TikTok @thequeenofmedia</t>
+          <t>TikTok @erinkatedolan (81.3k)</t>
         </is>
       </c>
       <c r="I49" s="6" t="inlineStr">
@@ -4616,14 +4616,14 @@
       </c>
       <c r="K49" s="6" t="inlineStr">
         <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="L49" s="6" t="inlineStr">
+        <is>
           <t>3.0</t>
         </is>
       </c>
-      <c r="L49" s="6" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
       <c r="M49" s="6" t="inlineStr">
         <is>
           <t>2.0</t>
@@ -4631,7 +4631,7 @@
       </c>
       <c r="N49" s="7" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O49" s="6" t="inlineStr">
@@ -4653,12 +4653,12 @@
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>erinkatedolan</t>
+          <t>Anthony Chico Reyes (Slot Machine Wins by Chico)</t>
         </is>
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>sports-betting</t>
+          <t>gambling-casino</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -4673,17 +4673,17 @@
       </c>
       <c r="F50" s="4" t="inlineStr">
         <is>
-          <t>~81.3k</t>
+          <t>~94k IG</t>
         </is>
       </c>
       <c r="G50" s="4" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>TikTok @erinkatedolan (81.3k)</t>
+          <t>IG https://instagram.com/slotmachinewinsbychico (94k)</t>
         </is>
       </c>
       <c r="I50" s="4" t="inlineStr">
@@ -4698,22 +4698,22 @@
       </c>
       <c r="K50" s="4" t="inlineStr">
         <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="L50" s="4" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M50" s="4" t="inlineStr">
+        <is>
           <t>2.0</t>
         </is>
       </c>
-      <c r="L50" s="4" t="inlineStr">
-        <is>
-          <t>3.0</t>
-        </is>
-      </c>
-      <c r="M50" s="4" t="inlineStr">
-        <is>
-          <t>2.0</t>
-        </is>
-      </c>
       <c r="N50" s="5" t="inlineStr">
         <is>
-          <t>sports-betting audience - core gambling fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
         </is>
       </c>
       <c r="O50" s="4" t="inlineStr">
@@ -4735,7 +4735,7 @@
       </c>
       <c r="B51" s="6" t="inlineStr">
         <is>
-          <t>Anthony Chico Reyes (Slot Machine Wins by Chico)</t>
+          <t>CasinoGrounds</t>
         </is>
       </c>
       <c r="C51" s="6" t="inlineStr">
@@ -4745,7 +4745,7 @@
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>micro</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
@@ -4755,17 +4755,17 @@
       </c>
       <c r="F51" s="6" t="inlineStr">
         <is>
-          <t>~94k IG</t>
+          <t>130,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="G51" s="6" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H51" s="7" t="inlineStr">
         <is>
-          <t>IG https://instagram.com/slotmachinewinsbychico (94k)</t>
+          <t>YouTube (CasinoGrounds)</t>
         </is>
       </c>
       <c r="I51" s="6" t="inlineStr">
@@ -4790,22 +4790,22 @@
       </c>
       <c r="M51" s="6" t="inlineStr">
         <is>
-          <t>2.0</t>
+          <t>3.0</t>
         </is>
       </c>
       <c r="N51" s="7" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; engaged micro/nano - sweet spot; contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; contact needs enrichment</t>
         </is>
       </c>
       <c r="O51" s="6" t="inlineStr">
         <is>
-          <t>$175-1,500</t>
+          <t>$1,500-6,000</t>
         </is>
       </c>
       <c r="P51" s="6" t="inlineStr">
         <is>
-          <t>$4,400-27,000</t>
+          <t>$27,000-90,000</t>
         </is>
       </c>
     </row>
@@ -5637,7 +5637,7 @@
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>Cheesur</t>
+          <t>Dima_wallhacks</t>
         </is>
       </c>
       <c r="C62" s="4" t="inlineStr">
@@ -5657,17 +5657,17 @@
       </c>
       <c r="F62" s="4" t="inlineStr">
         <is>
-          <t>~203k Kick ESTIMATE</t>
+          <t>203,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr">
         <is>
-          <t>https://kick.com/cheesur</t>
+          <t>https://www.youtube.com/@Dima_wallhacks</t>
         </is>
       </c>
       <c r="I62" s="4" t="inlineStr">
@@ -5719,7 +5719,7 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>PimpCSGO (Jacob Winneche)</t>
+          <t>Cheesur</t>
         </is>
       </c>
       <c r="C63" s="6" t="inlineStr">
@@ -5739,17 +5739,17 @@
       </c>
       <c r="F63" s="6" t="inlineStr">
         <is>
-          <t>~250k SUBS ESTIMATE</t>
+          <t>~203k Kick ESTIMATE</t>
         </is>
       </c>
       <c r="G63" s="6" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Kick</t>
         </is>
       </c>
       <c r="H63" s="7" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@PIMP</t>
+          <t>https://kick.com/cheesur</t>
         </is>
       </c>
       <c r="I63" s="6" t="inlineStr">
@@ -5801,7 +5801,7 @@
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>ProdigyDDK</t>
+          <t>PimpCSGO (Jacob Winneche)</t>
         </is>
       </c>
       <c r="C64" s="4" t="inlineStr">
@@ -5821,7 +5821,7 @@
       </c>
       <c r="F64" s="4" t="inlineStr">
         <is>
-          <t>~251-270k SUBS ESTIMATE (2026)</t>
+          <t>~250k SUBS ESTIMATE</t>
         </is>
       </c>
       <c r="G64" s="4" t="inlineStr">
@@ -5831,12 +5831,12 @@
       </c>
       <c r="H64" s="5" t="inlineStr">
         <is>
-          <t>YouTube https://www.youtube.com/@prodigyddk ; Instagram https://www.instagram.com/prodigy.ddk/ ; Twitch https://twitch.tv/prodigyddk</t>
+          <t>https://www.youtube.com/@PIMP</t>
         </is>
       </c>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>none (site prodigyddk.com)</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J64" s="4" t="inlineStr">
@@ -5883,7 +5883,7 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>Dima_wallhacks</t>
+          <t>ProdigyDDK</t>
         </is>
       </c>
       <c r="C65" s="6" t="inlineStr">
@@ -5903,7 +5903,7 @@
       </c>
       <c r="F65" s="6" t="inlineStr">
         <is>
-          <t>~406k SUBS ESTIMATE</t>
+          <t>258,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="G65" s="6" t="inlineStr">
@@ -5913,12 +5913,12 @@
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@Dima_wallhacks</t>
+          <t>YouTube https://www.youtube.com/@prodigyddk ; Instagram https://www.instagram.com/prodigy.ddk/ ; Twitch https://twitch.tv/prodigyddk</t>
         </is>
       </c>
       <c r="I65" s="6" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>none (site prodigyddk.com)</t>
         </is>
       </c>
       <c r="J65" s="6" t="inlineStr">
@@ -5965,7 +5965,7 @@
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>Maherco</t>
+          <t>Orangie</t>
         </is>
       </c>
       <c r="C66" s="4" t="inlineStr">
@@ -5975,7 +5975,7 @@
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="E66" s="4" t="inlineStr">
@@ -5985,17 +5985,17 @@
       </c>
       <c r="F66" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>355,663 X (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="G66" s="4" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>Twitch</t>
         </is>
       </c>
       <c r="H66" s="5" t="inlineStr">
         <is>
-          <t>https://kick.com/maherco</t>
+          <t>Twitch https://www.twitch.tv/orangieyt ; Kick https://kick.com/orangie ; X https://x.com/orangie ; YouTube https://www.youtube.com/watch?v=o2pvnwCtc0U</t>
         </is>
       </c>
       <c r="I66" s="4" t="inlineStr">
@@ -6005,19 +6005,19 @@
       </c>
       <c r="J66" s="4" t="inlineStr">
         <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="K66" s="4" t="inlineStr">
+        <is>
           <t>4.0</t>
         </is>
       </c>
-      <c r="K66" s="4" t="inlineStr">
+      <c r="L66" s="4" t="inlineStr">
         <is>
           <t>4.0</t>
         </is>
       </c>
-      <c r="L66" s="4" t="inlineStr">
-        <is>
-          <t>4.0</t>
-        </is>
-      </c>
       <c r="M66" s="4" t="inlineStr">
         <is>
           <t>2</t>
@@ -6030,12 +6030,12 @@
       </c>
       <c r="O66" s="4" t="inlineStr">
         <is>
-          <t>N/A ESTIMATE</t>
+          <t>$1,500-6,000</t>
         </is>
       </c>
       <c r="P66" s="4" t="inlineStr">
         <is>
-          <t>N/A ESTIMATE</t>
+          <t>$27,000-90,000</t>
         </is>
       </c>
     </row>
@@ -6047,7 +6047,7 @@
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>Renyan</t>
+          <t>Maherco</t>
         </is>
       </c>
       <c r="C67" s="6" t="inlineStr">
@@ -6072,12 +6072,12 @@
       </c>
       <c r="G67" s="6" t="inlineStr">
         <is>
-          <t>Twitch</t>
+          <t>Kick</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>https://www.twitch.tv/renyan</t>
+          <t>https://kick.com/maherco</t>
         </is>
       </c>
       <c r="I67" s="6" t="inlineStr">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>Curly (The Curly Fella)</t>
+          <t>Renyan</t>
         </is>
       </c>
       <c r="C68" s="4" t="inlineStr">
@@ -6154,12 +6154,12 @@
       </c>
       <c r="G68" s="4" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>Twitch</t>
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@thecurlyfella</t>
+          <t>https://www.twitch.tv/renyan</t>
         </is>
       </c>
       <c r="I68" s="4" t="inlineStr">
@@ -6211,7 +6211,7 @@
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>@culturekicks</t>
+          <t>Curly (The Curly Fella)</t>
         </is>
       </c>
       <c r="C69" s="6" t="inlineStr">
@@ -6241,7 +6241,7 @@
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@culturekicks</t>
+          <t>https://www.tiktok.com/@thecurlyfella</t>
         </is>
       </c>
       <c r="I69" s="6" t="inlineStr">
@@ -6293,7 +6293,7 @@
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>@soleloco</t>
+          <t>@culturekicks</t>
         </is>
       </c>
       <c r="C70" s="4" t="inlineStr">
@@ -6323,7 +6323,7 @@
       </c>
       <c r="H70" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@soleloco</t>
+          <t>https://www.tiktok.com/@culturekicks</t>
         </is>
       </c>
       <c r="I70" s="4" t="inlineStr">
@@ -6375,7 +6375,7 @@
       </c>
       <c r="B71" s="6" t="inlineStr">
         <is>
-          <t>@air.jumps.official</t>
+          <t>@soleloco</t>
         </is>
       </c>
       <c r="C71" s="6" t="inlineStr">
@@ -6405,7 +6405,7 @@
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@air.jumps.official</t>
+          <t>https://www.tiktok.com/@soleloco</t>
         </is>
       </c>
       <c r="I71" s="6" t="inlineStr">
@@ -6457,7 +6457,7 @@
       </c>
       <c r="B72" s="4" t="inlineStr">
         <is>
-          <t>@ioannalaou</t>
+          <t>@air.jumps.official</t>
         </is>
       </c>
       <c r="C72" s="4" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="H72" s="5" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@ioannalaou</t>
+          <t>https://www.tiktok.com/@air.jumps.official</t>
         </is>
       </c>
       <c r="I72" s="4" t="inlineStr">
@@ -6539,7 +6539,7 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>csgo.gambling</t>
+          <t>@ioannalaou</t>
         </is>
       </c>
       <c r="C73" s="6" t="inlineStr">
@@ -6569,7 +6569,7 @@
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@csgo.gambling</t>
+          <t>https://www.tiktok.com/@ioannalaou</t>
         </is>
       </c>
       <c r="I73" s="6" t="inlineStr">
@@ -6621,7 +6621,7 @@
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>dizzydankss (DizzyDanks24)</t>
+          <t>csgo.gambling</t>
         </is>
       </c>
       <c r="C74" s="4" t="inlineStr">
@@ -6651,7 +6651,7 @@
       </c>
       <c r="H74" s="5" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@dizzydankss</t>
+          <t>TikTok https://www.tiktok.com/@csgo.gambling</t>
         </is>
       </c>
       <c r="I74" s="4" t="inlineStr">
@@ -6703,7 +6703,7 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>hypedropbalotelli</t>
+          <t>dizzydankss (DizzyDanks24)</t>
         </is>
       </c>
       <c r="C75" s="6" t="inlineStr">
@@ -6733,7 +6733,7 @@
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@hypedropbalotelli</t>
+          <t>TikTok https://www.tiktok.com/@dizzydankss</t>
         </is>
       </c>
       <c r="I75" s="6" t="inlineStr">
@@ -6785,7 +6785,7 @@
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>kelvinmboik</t>
+          <t>hypedropbalotelli</t>
         </is>
       </c>
       <c r="C76" s="4" t="inlineStr">
@@ -6815,7 +6815,7 @@
       </c>
       <c r="H76" s="5" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@kelvinmboik</t>
+          <t>TikTok https://www.tiktok.com/@hypedropbalotelli</t>
         </is>
       </c>
       <c r="I76" s="4" t="inlineStr">
@@ -6867,7 +6867,7 @@
       </c>
       <c r="B77" s="6" t="inlineStr">
         <is>
-          <t>laceduphollywood</t>
+          <t>kelvinmboik</t>
         </is>
       </c>
       <c r="C77" s="6" t="inlineStr">
@@ -6892,17 +6892,17 @@
       </c>
       <c r="G77" s="6" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>Instagram https://www.instagram.com/laceduphollywood/</t>
+          <t>TikTok https://www.tiktok.com/@kelvinmboik</t>
         </is>
       </c>
       <c r="I77" s="6" t="inlineStr">
         <is>
-          <t>retail store</t>
+          <t>none</t>
         </is>
       </c>
       <c r="J77" s="6" t="inlineStr">
@@ -6949,7 +6949,7 @@
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>OnlyCrunchy</t>
+          <t>laceduphollywood</t>
         </is>
       </c>
       <c r="C78" s="4" t="inlineStr">
@@ -6974,17 +6974,17 @@
       </c>
       <c r="G78" s="4" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="H78" s="5" t="inlineStr">
         <is>
-          <t>X https://x.com/onlycrunchy</t>
+          <t>Instagram https://www.instagram.com/laceduphollywood/</t>
         </is>
       </c>
       <c r="I78" s="4" t="inlineStr">
         <is>
-          <t>none</t>
+          <t>retail store</t>
         </is>
       </c>
       <c r="J78" s="4" t="inlineStr">
@@ -7031,7 +7031,7 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>pizza_god1 (Kody Garrett)</t>
+          <t>OnlyCrunchy</t>
         </is>
       </c>
       <c r="C79" s="6" t="inlineStr">
@@ -7056,12 +7056,12 @@
       </c>
       <c r="G79" s="6" t="inlineStr">
         <is>
-          <t>TikTok</t>
+          <t>X</t>
         </is>
       </c>
       <c r="H79" s="7" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@pizza_god1</t>
+          <t>X https://x.com/onlycrunchy</t>
         </is>
       </c>
       <c r="I79" s="6" t="inlineStr">
@@ -7113,7 +7113,7 @@
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>quickhypedrop</t>
+          <t>pizza_god1 (Kody Garrett)</t>
         </is>
       </c>
       <c r="C80" s="4" t="inlineStr">
@@ -7143,7 +7143,7 @@
       </c>
       <c r="H80" s="5" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@quickhypedrop</t>
+          <t>TikTok https://www.tiktok.com/@pizza_god1</t>
         </is>
       </c>
       <c r="I80" s="4" t="inlineStr">
@@ -7195,7 +7195,7 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>rillabox.openings</t>
+          <t>quickhypedrop</t>
         </is>
       </c>
       <c r="C81" s="6" t="inlineStr">
@@ -7225,7 +7225,7 @@
       </c>
       <c r="H81" s="7" t="inlineStr">
         <is>
-          <t>TikTok https://www.tiktok.com/@rillabox.openings</t>
+          <t>TikTok https://www.tiktok.com/@quickhypedrop</t>
         </is>
       </c>
       <c r="I81" s="6" t="inlineStr">
@@ -7277,7 +7277,7 @@
       </c>
       <c r="B82" s="4" t="inlineStr">
         <is>
-          <t>twitch.tvkushti_ (kushti_)</t>
+          <t>rillabox.openings</t>
         </is>
       </c>
       <c r="C82" s="4" t="inlineStr">
@@ -7302,12 +7302,12 @@
       </c>
       <c r="G82" s="4" t="inlineStr">
         <is>
-          <t>Instagram</t>
+          <t>TikTok</t>
         </is>
       </c>
       <c r="H82" s="5" t="inlineStr">
         <is>
-          <t>Instagram https://www.instagram.com/twitch.tvkushti_/</t>
+          <t>TikTok https://www.tiktok.com/@rillabox.openings</t>
         </is>
       </c>
       <c r="I82" s="4" t="inlineStr">
@@ -7359,7 +7359,7 @@
       </c>
       <c r="B83" s="6" t="inlineStr">
         <is>
-          <t>@harrisonevel</t>
+          <t>twitch.tvkushti_ (kushti_)</t>
         </is>
       </c>
       <c r="C83" s="6" t="inlineStr">
@@ -7387,7 +7387,11 @@
           <t>Instagram</t>
         </is>
       </c>
-      <c r="H83" s="7" t="inlineStr"/>
+      <c r="H83" s="7" t="inlineStr">
+        <is>
+          <t>Instagram https://www.instagram.com/twitch.tvkushti_/</t>
+        </is>
+      </c>
       <c r="I83" s="6" t="inlineStr">
         <is>
           <t>none</t>
@@ -7437,7 +7441,7 @@
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>@yankeekicks</t>
+          <t>@harrisonevel</t>
         </is>
       </c>
       <c r="C84" s="4" t="inlineStr">
@@ -7462,7 +7466,7 @@
       </c>
       <c r="G84" s="4" t="inlineStr">
         <is>
-          <t>Instagram/YouTube</t>
+          <t>Instagram</t>
         </is>
       </c>
       <c r="H84" s="5" t="inlineStr"/>
@@ -7515,7 +7519,7 @@
       </c>
       <c r="B85" s="6" t="inlineStr">
         <is>
-          <t>ArrowCS</t>
+          <t>@yankeekicks</t>
         </is>
       </c>
       <c r="C85" s="6" t="inlineStr">
@@ -7540,7 +7544,7 @@
       </c>
       <c r="G85" s="6" t="inlineStr">
         <is>
-          <t>Twitch</t>
+          <t>Instagram/YouTube</t>
         </is>
       </c>
       <c r="H85" s="7" t="inlineStr"/>
@@ -7593,7 +7597,7 @@
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>Devon Gard</t>
+          <t>ArrowCS</t>
         </is>
       </c>
       <c r="C86" s="4" t="inlineStr">
@@ -7618,7 +7622,7 @@
       </c>
       <c r="G86" s="4" t="inlineStr">
         <is>
-          <t>YouTube/LinkedIn</t>
+          <t>Twitch</t>
         </is>
       </c>
       <c r="H86" s="5" t="inlineStr"/>
@@ -7671,7 +7675,7 @@
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>megalodon888</t>
+          <t>Devon Gard</t>
         </is>
       </c>
       <c r="C87" s="6" t="inlineStr">
@@ -7696,7 +7700,7 @@
       </c>
       <c r="G87" s="6" t="inlineStr">
         <is>
-          <t>Twitch/Kick</t>
+          <t>YouTube/LinkedIn</t>
         </is>
       </c>
       <c r="H87" s="7" t="inlineStr"/>
@@ -7749,17 +7753,17 @@
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>Raja Richter (The Big Jackpot)</t>
+          <t>megalodon888</t>
         </is>
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>gambling-casino</t>
+          <t>case-opening/mystery-box</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>unknown</t>
         </is>
       </c>
       <c r="E88" s="4" t="inlineStr">
@@ -7769,19 +7773,15 @@
       </c>
       <c r="F88" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="G88" s="4" t="inlineStr">
         <is>
-          <t>YouTube</t>
-        </is>
-      </c>
-      <c r="H88" s="5" t="inlineStr">
-        <is>
-          <t>YouTube @TheBigJackpot ; IG @thebigjackpot</t>
-        </is>
-      </c>
+          <t>Twitch/Kick</t>
+        </is>
+      </c>
+      <c r="H88" s="5" t="inlineStr"/>
       <c r="I88" s="4" t="inlineStr">
         <is>
           <t>none</t>
@@ -7794,32 +7794,32 @@
       </c>
       <c r="K88" s="4" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="L88" s="4" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>4.0</t>
         </is>
       </c>
       <c r="M88" s="4" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>2</t>
         </is>
       </c>
       <c r="N88" s="5" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; macro reach (higher cost); contact needs enrichment</t>
+          <t>real-money case/box gambling - core gambling fit; contact needs enrichment</t>
         </is>
       </c>
       <c r="O88" s="4" t="inlineStr">
         <is>
-          <t>$6,000-30,000</t>
+          <t>N/A ESTIMATE</t>
         </is>
       </c>
       <c r="P88" s="4" t="inlineStr">
         <is>
-          <t>$90,000-700,000+</t>
+          <t>N/A ESTIMATE</t>
         </is>
       </c>
     </row>
@@ -7831,7 +7831,7 @@
       </c>
       <c r="B89" s="6" t="inlineStr">
         <is>
-          <t>Lady Luck HQ</t>
+          <t>Pompsie Slots</t>
         </is>
       </c>
       <c r="C89" s="6" t="inlineStr">
@@ -7841,7 +7841,7 @@
       </c>
       <c r="D89" s="6" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="E89" s="6" t="inlineStr">
@@ -7851,7 +7851,7 @@
       </c>
       <c r="F89" s="6" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="G89" s="6" t="inlineStr">
@@ -7861,7 +7861,7 @@
       </c>
       <c r="H89" s="7" t="inlineStr">
         <is>
-          <t>YouTube @LadyLuckHQ</t>
+          <t>YouTube (Pompsie)</t>
         </is>
       </c>
       <c r="I89" s="6" t="inlineStr">
@@ -7886,22 +7886,22 @@
       </c>
       <c r="M89" s="6" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="N89" s="7" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; macro reach (higher cost); contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; contact needs enrichment</t>
         </is>
       </c>
       <c r="O89" s="6" t="inlineStr">
         <is>
-          <t>$6,000-30,000</t>
+          <t>$1,500-6,000</t>
         </is>
       </c>
       <c r="P89" s="6" t="inlineStr">
         <is>
-          <t>$90,000-700,000+</t>
+          <t>$27,000-90,000</t>
         </is>
       </c>
     </row>
@@ -7913,7 +7913,7 @@
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>NG Slot</t>
+          <t>PokerMetarb</t>
         </is>
       </c>
       <c r="C90" s="4" t="inlineStr">
@@ -7923,7 +7923,7 @@
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="E90" s="4" t="inlineStr">
@@ -7933,7 +7933,7 @@
       </c>
       <c r="F90" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="G90" s="4" t="inlineStr">
@@ -7943,7 +7943,7 @@
       </c>
       <c r="H90" s="5" t="inlineStr">
         <is>
-          <t>YouTube @NGSlot</t>
+          <t>YouTube (PokerMetarb)</t>
         </is>
       </c>
       <c r="I90" s="4" t="inlineStr">
@@ -7968,22 +7968,22 @@
       </c>
       <c r="M90" s="4" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="N90" s="5" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; macro reach (higher cost); contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; contact needs enrichment</t>
         </is>
       </c>
       <c r="O90" s="4" t="inlineStr">
         <is>
-          <t>$6,000-30,000</t>
+          <t>$1,500-6,000</t>
         </is>
       </c>
       <c r="P90" s="4" t="inlineStr">
         <is>
-          <t>$90,000-700,000+</t>
+          <t>$27,000-90,000</t>
         </is>
       </c>
     </row>
@@ -7995,7 +7995,7 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>Mr. Hand Pay</t>
+          <t>CasinoDaddy</t>
         </is>
       </c>
       <c r="C91" s="6" t="inlineStr">
@@ -8020,12 +8020,12 @@
       </c>
       <c r="G91" s="6" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Twitch</t>
         </is>
       </c>
       <c r="H91" s="7" t="inlineStr">
         <is>
-          <t>YouTube @MrHandPay</t>
+          <t>Twitch https://twitch.tv/casinodaddy</t>
         </is>
       </c>
       <c r="I91" s="6" t="inlineStr">
@@ -8077,7 +8077,7 @@
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>Pompsie Slots</t>
+          <t>Taour (Noamane Boukhari)</t>
         </is>
       </c>
       <c r="C92" s="4" t="inlineStr">
@@ -8097,17 +8097,17 @@
       </c>
       <c r="F92" s="4" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>mid-macro</t>
         </is>
       </c>
       <c r="G92" s="4" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Kick</t>
         </is>
       </c>
       <c r="H92" s="5" t="inlineStr">
         <is>
-          <t>YouTube (Pompsie)</t>
+          <t>Kick (Taour)</t>
         </is>
       </c>
       <c r="I92" s="4" t="inlineStr">
@@ -8159,7 +8159,7 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>PokerMetarb</t>
+          <t>Tiagovski</t>
         </is>
       </c>
       <c r="C93" s="6" t="inlineStr">
@@ -8184,12 +8184,12 @@
       </c>
       <c r="G93" s="6" t="inlineStr">
         <is>
-          <t>YouTube</t>
+          <t>Kick</t>
         </is>
       </c>
       <c r="H93" s="7" t="inlineStr">
         <is>
-          <t>YouTube (PokerMetarb)</t>
+          <t>Kick/Twitch @Tiagovski555</t>
         </is>
       </c>
       <c r="I93" s="6" t="inlineStr">
@@ -8241,7 +8241,7 @@
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>CasinoDaddy</t>
+          <t>teufeurs</t>
         </is>
       </c>
       <c r="C94" s="4" t="inlineStr">
@@ -8251,7 +8251,7 @@
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="E94" s="4" t="inlineStr">
@@ -8261,7 +8261,7 @@
       </c>
       <c r="F94" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="G94" s="4" t="inlineStr">
@@ -8271,7 +8271,7 @@
       </c>
       <c r="H94" s="5" t="inlineStr">
         <is>
-          <t>Twitch https://twitch.tv/casinodaddy</t>
+          <t>Twitch @teufeurs</t>
         </is>
       </c>
       <c r="I94" s="4" t="inlineStr">
@@ -8296,22 +8296,22 @@
       </c>
       <c r="M94" s="4" t="inlineStr">
         <is>
-          <t>3.0</t>
+          <t>2.0</t>
         </is>
       </c>
       <c r="N94" s="5" t="inlineStr">
         <is>
-          <t>real-money gambling/casino audience - TOP GemBreak fit; macro reach (higher cost); contact needs enrichment</t>
+          <t>real-money gambling/casino audience - TOP GemBreak fit; contact needs enrichment</t>
         </is>
       </c>
       <c r="O94" s="4" t="inlineStr">
         <is>
-          <t>$6,000-30,000</t>
+          <t>$1,500-6,000</t>
         </is>
       </c>
       <c r="P94" s="4" t="inlineStr">
         <is>
-          <t>$90,000-700,000+</t>
+          <t>$27,000-90,000</t>
         </is>
       </c>
     </row>
@@ -8323,7 +8323,7 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>Taour (Noamane Boukhari)</t>
+          <t>YoutubeVLR</t>
         </is>
       </c>
       <c r="C95" s="6" t="inlineStr">
@@ -8343,17 +8343,17 @@
       </c>
       <c r="F95" s="6" t="inlineStr">
         <is>
-          <t>mid-macro</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="G95" s="6" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H95" s="7" t="inlineStr">
         <is>
-          <t>Kick (Taour)</t>
+          <t>YouTube (VLR)</t>
         </is>
       </c>
       <c r="I95" s="6" t="inlineStr">
@@ -8405,7 +8405,7 @@
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>Tiagovski</t>
+          <t>All Casino Action</t>
         </is>
       </c>
       <c r="C96" s="4" t="inlineStr">
@@ -8430,12 +8430,12 @@
       </c>
       <c r="G96" s="4" t="inlineStr">
         <is>
-          <t>Kick</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H96" s="5" t="inlineStr">
         <is>
-          <t>Kick/Twitch @Tiagovski555</t>
+          <t>YouTube (All Casino Action)</t>
         </is>
       </c>
       <c r="I96" s="4" t="inlineStr">
@@ -8487,7 +8487,7 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>teufeurs</t>
+          <t>Chipmonkz Slots</t>
         </is>
       </c>
       <c r="C97" s="6" t="inlineStr">
@@ -8512,12 +8512,12 @@
       </c>
       <c r="G97" s="6" t="inlineStr">
         <is>
-          <t>Twitch</t>
+          <t>YouTube</t>
         </is>
       </c>
       <c r="H97" s="7" t="inlineStr">
         <is>
-          <t>Twitch @teufeurs</t>
+          <t>YouTube (Chipmonkz)</t>
         </is>
       </c>
       <c r="I97" s="6" t="inlineStr">
@@ -8569,7 +8569,7 @@
       </c>
       <c r="B98" s="4" t="inlineStr">
         <is>
-          <t>YoutubeVLR</t>
+          <t>Toaster (Toaster Gambles)</t>
         </is>
       </c>
       <c r="C98" s="4" t="inlineStr">
@@ -8599,7 +8599,7 @@
       </c>
       <c r="H98" s="5" t="inlineStr">
         <is>
-          <t>YouTube (VLR)</t>
+          <t>YouTube/Kick (Toaster)</t>
         </is>
       </c>
       <c r="I98" s="4" t="inlineStr">
@@ -8651,7 +8651,7 @@
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>All Casino Action</t>
+          <t>Cabrzy</t>
         </is>
       </c>
       <c r="C99" s="6" t="inlineStr">
@@ -8681,7 +8681,7 @@
       </c>
       <c r="H99" s="7" t="inlineStr">
         <is>
-          <t>YouTube (All Casino Action)</t>
+          <t>YouTube/Kick (Cabrzy)</t>
         </is>
       </c>
       <c r="I99" s="6" t="inlineStr">
@@ -8733,7 +8733,7 @@
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>Chipmonkz Slots</t>
+          <t>TactPlaysGames</t>
         </is>
       </c>
       <c r="C100" s="4" t="inlineStr">
@@ -8763,7 +8763,7 @@
       </c>
       <c r="H100" s="5" t="inlineStr">
         <is>
-          <t>YouTube (Chipmonkz)</t>
+          <t>YouTube (Tact)</t>
         </is>
       </c>
       <c r="I100" s="4" t="inlineStr">
@@ -8815,7 +8815,7 @@
       </c>
       <c r="B101" s="6" t="inlineStr">
         <is>
-          <t>Toaster (Toaster Gambles)</t>
+          <t>The Bandit (NightRush/Slot Video)</t>
         </is>
       </c>
       <c r="C101" s="6" t="inlineStr">
@@ -8845,7 +8845,7 @@
       </c>
       <c r="H101" s="7" t="inlineStr">
         <is>
-          <t>YouTube/Kick (Toaster)</t>
+          <t>YouTube (The Bandit)</t>
         </is>
       </c>
       <c r="I101" s="6" t="inlineStr">
@@ -9039,12 +9039,12 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>60,625 X (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr"/>
@@ -9081,17 +9081,17 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>modash/WSJ coverage</t>
+          <t>modash/WSJ coverage +LunarCrush</t>
         </is>
       </c>
       <c r="P2" s="4" t="inlineStr">
         <is>
-          <t>N/A ESTIMATE</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="Q2" s="4" t="inlineStr">
         <is>
-          <t>N/A ESTIMATE</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr">
@@ -10015,7 +10015,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>680,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -10057,7 +10057,7 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P14" s="4" t="inlineStr">
@@ -10095,7 +10095,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>~1M+ ESTIMATE</t>
+          <t>1,610,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -10137,7 +10137,7 @@
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P15" s="6" t="inlineStr">
@@ -10175,7 +10175,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>1,200,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -10217,7 +10217,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P16" s="4" t="inlineStr">
@@ -10335,7 +10335,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>1,260,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -10377,7 +10377,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P18" s="4" t="inlineStr">
@@ -10495,7 +10495,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>1,140,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -10537,7 +10537,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P20" s="4" t="inlineStr">
@@ -11859,7 +11859,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>130,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -11901,7 +11901,7 @@
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P37" s="6" t="inlineStr">
@@ -12099,7 +12099,7 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>mid-macro</t>
+          <t>318,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
@@ -12141,7 +12141,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P40" s="4" t="inlineStr">
@@ -12339,12 +12339,12 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>78,700 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr"/>
@@ -12381,17 +12381,17 @@
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P43" s="6" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="Q43" s="6" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
       <c r="R43" s="7" t="inlineStr"/>
@@ -16153,7 +16153,7 @@
       </c>
       <c r="O90" s="4" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P90" s="4" t="inlineStr">
@@ -16233,7 +16233,7 @@
       </c>
       <c r="O91" s="6" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P91" s="6" t="inlineStr">
@@ -16313,7 +16313,7 @@
       </c>
       <c r="O92" s="4" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P92" s="4" t="inlineStr">
@@ -16393,7 +16393,7 @@
       </c>
       <c r="O93" s="6" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P93" s="6" t="inlineStr">
@@ -16473,7 +16473,7 @@
       </c>
       <c r="O94" s="4" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P94" s="4" t="inlineStr">
@@ -16557,7 +16557,7 @@
       </c>
       <c r="O95" s="6" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P95" s="6" t="inlineStr">
@@ -17365,7 +17365,7 @@
       </c>
       <c r="O105" s="6" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P105" s="6" t="inlineStr">
@@ -22475,7 +22475,7 @@
       </c>
       <c r="E169" s="6" t="inlineStr">
         <is>
-          <t>~1.74M YT / 419k IG</t>
+          <t>2,060,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F169" s="6" t="inlineStr">
@@ -22521,7 +22521,7 @@
       </c>
       <c r="O169" s="6" t="inlineStr">
         <is>
-          <t>favikon/feedspot/press</t>
+          <t>favikon/feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P169" s="6" t="inlineStr">
@@ -22559,7 +22559,7 @@
       </c>
       <c r="E170" s="4" t="inlineStr">
         <is>
-          <t>~600k+ YT</t>
+          <t>1,490,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F170" s="4" t="inlineStr">
@@ -22605,7 +22605,7 @@
       </c>
       <c r="O170" s="4" t="inlineStr">
         <is>
-          <t>favikon/feedspot/press</t>
+          <t>favikon/feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P170" s="4" t="inlineStr">
@@ -22643,7 +22643,7 @@
       </c>
       <c r="E171" s="6" t="inlineStr">
         <is>
-          <t>~300-600k YT</t>
+          <t>599,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F171" s="6" t="inlineStr">
@@ -22685,7 +22685,7 @@
       </c>
       <c r="O171" s="6" t="inlineStr">
         <is>
-          <t>favikon/feedspot/press</t>
+          <t>favikon/feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P171" s="6" t="inlineStr">
@@ -23623,7 +23623,7 @@
       </c>
       <c r="E183" s="6" t="inlineStr">
         <is>
-          <t>~334k</t>
+          <t>~334k YT ESTIMATE</t>
         </is>
       </c>
       <c r="F183" s="6" t="inlineStr">
@@ -24523,7 +24523,7 @@
       </c>
       <c r="E194" s="4" t="inlineStr">
         <is>
-          <t>macro ESTIMATE</t>
+          <t>1,170,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F194" s="4" t="inlineStr">
@@ -24569,7 +24569,7 @@
       </c>
       <c r="O194" s="4" t="inlineStr">
         <is>
-          <t>press</t>
+          <t>press +LunarCrush</t>
         </is>
       </c>
       <c r="P194" s="4" t="inlineStr">
@@ -25175,7 +25175,7 @@
       </c>
       <c r="E202" s="4" t="inlineStr">
         <is>
-          <t>macro &gt;&gt;1M</t>
+          <t>1,004,182 X (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F202" s="4" t="inlineStr">
@@ -25511,7 +25511,7 @@
       </c>
       <c r="E206" s="4" t="inlineStr">
         <is>
-          <t>macro (multi-M)</t>
+          <t>675,558 X (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F206" s="4" t="inlineStr">
@@ -25679,12 +25679,12 @@
       </c>
       <c r="E208" s="4" t="inlineStr">
         <is>
-          <t>~553k SUBS ESTIMATE</t>
+          <t>549,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F208" s="4" t="inlineStr">
         <is>
-          <t>mid-macro</t>
+          <t>macro</t>
         </is>
       </c>
       <c r="G208" s="4" t="inlineStr"/>
@@ -25763,12 +25763,12 @@
       </c>
       <c r="E209" s="6" t="inlineStr">
         <is>
-          <t>N/A (crowded namespace)</t>
+          <t>355,663 X (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F209" s="6" t="inlineStr">
         <is>
-          <t>mid-macro</t>
+          <t>mid</t>
         </is>
       </c>
       <c r="G209" s="6" t="inlineStr"/>
@@ -25814,12 +25814,12 @@
       </c>
       <c r="P209" s="6" t="inlineStr">
         <is>
-          <t>$6,000-30,000</t>
+          <t>$1,500-6,000</t>
         </is>
       </c>
       <c r="Q209" s="6" t="inlineStr">
         <is>
-          <t>$90,000-700,000+</t>
+          <t>$27,000-90,000</t>
         </is>
       </c>
       <c r="R209" s="7" t="inlineStr"/>
@@ -25847,12 +25847,12 @@
       </c>
       <c r="E210" s="4" t="inlineStr">
         <is>
-          <t>~535-559k SUBS ESTIMATE (2026)</t>
+          <t>573,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F210" s="4" t="inlineStr">
         <is>
-          <t>mid-macro</t>
+          <t>macro</t>
         </is>
       </c>
       <c r="G210" s="4" t="inlineStr"/>
@@ -25931,12 +25931,12 @@
       </c>
       <c r="E211" s="6" t="inlineStr">
         <is>
-          <t>~535k SUBS ESTIMATE</t>
+          <t>538,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F211" s="6" t="inlineStr">
         <is>
-          <t>mid-macro</t>
+          <t>macro</t>
         </is>
       </c>
       <c r="G211" s="6" t="inlineStr"/>
@@ -26099,12 +26099,12 @@
       </c>
       <c r="E213" s="6" t="inlineStr">
         <is>
-          <t>~526k SUBS ESTIMATE</t>
+          <t>529,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F213" s="6" t="inlineStr">
         <is>
-          <t>mid-macro</t>
+          <t>macro</t>
         </is>
       </c>
       <c r="G213" s="6" t="inlineStr"/>
@@ -26183,7 +26183,7 @@
       </c>
       <c r="E214" s="4" t="inlineStr">
         <is>
-          <t>~406k SUBS ESTIMATE</t>
+          <t>203,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F214" s="4" t="inlineStr">
@@ -26267,7 +26267,7 @@
       </c>
       <c r="E215" s="6" t="inlineStr">
         <is>
-          <t>~251-270k SUBS ESTIMATE (2026)</t>
+          <t>258,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F215" s="6" t="inlineStr">
@@ -26855,12 +26855,12 @@
       </c>
       <c r="E222" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>5,930 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F222" s="4" t="inlineStr">
         <is>
-          <t>micro-mid</t>
+          <t>nano</t>
         </is>
       </c>
       <c r="G222" s="4" t="inlineStr"/>
@@ -26906,12 +26906,12 @@
       </c>
       <c r="P222" s="4" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$50-300</t>
         </is>
       </c>
       <c r="Q222" s="4" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$450-4,400</t>
         </is>
       </c>
       <c r="R222" s="5" t="inlineStr"/>
@@ -26939,12 +26939,12 @@
       </c>
       <c r="E223" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>2,850 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F223" s="6" t="inlineStr">
         <is>
-          <t>micro-mid</t>
+          <t>nano</t>
         </is>
       </c>
       <c r="G223" s="6" t="inlineStr"/>
@@ -26990,12 +26990,12 @@
       </c>
       <c r="P223" s="6" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$50-300</t>
         </is>
       </c>
       <c r="Q223" s="6" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$450-4,400</t>
         </is>
       </c>
       <c r="R223" s="7" t="inlineStr"/>
@@ -27023,12 +27023,12 @@
       </c>
       <c r="E224" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>453 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F224" s="4" t="inlineStr">
         <is>
-          <t>micro-mid</t>
+          <t>nano</t>
         </is>
       </c>
       <c r="G224" s="4" t="inlineStr"/>
@@ -27074,12 +27074,12 @@
       </c>
       <c r="P224" s="4" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$50-300</t>
         </is>
       </c>
       <c r="Q224" s="4" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$450-4,400</t>
         </is>
       </c>
       <c r="R224" s="5" t="inlineStr"/>
@@ -27107,12 +27107,12 @@
       </c>
       <c r="E225" s="6" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>5,880 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F225" s="6" t="inlineStr">
         <is>
-          <t>micro-mid</t>
+          <t>nano</t>
         </is>
       </c>
       <c r="G225" s="6" t="inlineStr"/>
@@ -27158,12 +27158,12 @@
       </c>
       <c r="P225" s="6" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$50-300</t>
         </is>
       </c>
       <c r="Q225" s="6" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$450-4,400</t>
         </is>
       </c>
       <c r="R225" s="7" t="inlineStr"/>
@@ -27779,7 +27779,7 @@
       </c>
       <c r="E233" s="6" t="inlineStr">
         <is>
-          <t>Kick ~24.2k (Sept-2025 snippet)</t>
+          <t>12,801 X (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F233" s="6" t="inlineStr">
@@ -30574,12 +30574,12 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>60,625 X (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>unknown</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="G2" s="4" t="inlineStr"/>
@@ -30616,17 +30616,17 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>modash/WSJ coverage</t>
+          <t>modash/WSJ coverage +LunarCrush</t>
         </is>
       </c>
       <c r="P2" s="4" t="inlineStr">
         <is>
-          <t>N/A ESTIMATE</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="Q2" s="4" t="inlineStr">
         <is>
-          <t>N/A ESTIMATE</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
       <c r="R2" s="5" t="inlineStr">
@@ -31550,7 +31550,7 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>680,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F14" s="4" t="inlineStr">
@@ -31592,7 +31592,7 @@
       </c>
       <c r="O14" s="4" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P14" s="4" t="inlineStr">
@@ -31630,7 +31630,7 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>~1M+ ESTIMATE</t>
+          <t>1,610,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
@@ -31672,7 +31672,7 @@
       </c>
       <c r="O15" s="6" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P15" s="6" t="inlineStr">
@@ -31710,7 +31710,7 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>1,200,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F16" s="4" t="inlineStr">
@@ -31752,7 +31752,7 @@
       </c>
       <c r="O16" s="4" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P16" s="4" t="inlineStr">
@@ -31870,7 +31870,7 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>1,260,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F18" s="4" t="inlineStr">
@@ -31912,7 +31912,7 @@
       </c>
       <c r="O18" s="4" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P18" s="4" t="inlineStr">
@@ -32030,7 +32030,7 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>macro</t>
+          <t>1,140,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F20" s="4" t="inlineStr">
@@ -32072,7 +32072,7 @@
       </c>
       <c r="O20" s="4" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P20" s="4" t="inlineStr">
@@ -33394,7 +33394,7 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>130,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -33436,7 +33436,7 @@
       </c>
       <c r="O37" s="6" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P37" s="6" t="inlineStr">
@@ -33634,7 +33634,7 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>mid-macro</t>
+          <t>318,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F40" s="4" t="inlineStr">
@@ -33676,7 +33676,7 @@
       </c>
       <c r="O40" s="4" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P40" s="4" t="inlineStr">
@@ -33874,12 +33874,12 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>78,700 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>mid</t>
+          <t>micro</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr"/>
@@ -33916,17 +33916,17 @@
       </c>
       <c r="O43" s="6" t="inlineStr">
         <is>
-          <t>StreamRollers/Feedspot/press</t>
+          <t>StreamRollers/Feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P43" s="6" t="inlineStr">
         <is>
-          <t>$1,500-6,000</t>
+          <t>$175-1,500</t>
         </is>
       </c>
       <c r="Q43" s="6" t="inlineStr">
         <is>
-          <t>$27,000-90,000</t>
+          <t>$4,400-27,000</t>
         </is>
       </c>
       <c r="R43" s="7" t="inlineStr"/>
@@ -37861,7 +37861,7 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>~1.74M YT / 419k IG</t>
+          <t>2,060,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F3" s="6" t="inlineStr">
@@ -37907,7 +37907,7 @@
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
-          <t>favikon/feedspot/press</t>
+          <t>favikon/feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P3" s="6" t="inlineStr">
@@ -37945,7 +37945,7 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>~600k+ YT</t>
+          <t>1,490,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
@@ -37991,7 +37991,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>favikon/feedspot/press</t>
+          <t>favikon/feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P4" s="4" t="inlineStr">
@@ -38029,7 +38029,7 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>~300-600k YT</t>
+          <t>599,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
@@ -38071,7 +38071,7 @@
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
-          <t>favikon/feedspot/press</t>
+          <t>favikon/feedspot/press +LunarCrush</t>
         </is>
       </c>
       <c r="P5" s="6" t="inlineStr">
@@ -39009,7 +39009,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>~334k</t>
+          <t>~334k YT ESTIMATE</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -39909,7 +39909,7 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>macro ESTIMATE</t>
+          <t>1,170,000 YT (LunarCrush 2026-07-19)</t>
         </is>
       </c>
       <c r="F28" s="4" t="inlineStr">
@@ -39955,7 +39955,7 @@
       </c>
       <c r="O28" s="4" t="inlineStr">
         <is>
-          <t>press</t>
+          <t>press +LunarCrush</t>
         </is>
       </c>
       <c r="P28" s="4" t="inlineStr">
@@ -40646,7 +40646,7 @@
       </c>
       <c r="O2" s="4" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P2" s="4" t="inlineStr">
@@ -40726,7 +40726,7 @@
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P3" s="6" t="inlineStr">
@@ -40806,7 +40806,7 @@
       </c>
       <c r="O4" s="4" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P4" s="4" t="inlineStr">
@@ -40886,7 +40886,7 @@
       </c>
       <c r="O5" s="6" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P5" s="6" t="inlineStr">
@@ -40966,7 +40966,7 @@
       </c>
       <c r="O6" s="4" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P6" s="4" t="inlineStr">
@@ -41050,7 +41050,7 @@
       </c>
       <c r="O7" s="6" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P7" s="6" t="inlineStr">
@@ -41858,7 +41858,7 @@
       </c>
       <c r="O17" s="6" t="inlineStr">
         <is>
-          <t>feedspot/socialveins/press</t>
+          <t>feedspot/socialveins/press +LunarCrush</t>
         </is>
       </c>
       <c r="P17" s="6" t="inlineStr">

</xml_diff>